<commit_message>
fixed bug in build_476_context_counts.R
</commit_message>
<xml_diff>
--- a/development/one_file_rosetta_output/SP48008_context_counts.xlsx
+++ b/development/one_file_rosetta_output/SP48008_context_counts.xlsx
@@ -393,7 +393,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
@@ -476,7 +476,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GT</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -530,7 +549,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AC</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -558,33 +596,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TT</t>
+            <t>GA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -612,38 +669,57 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GC</t>
+            <t>TT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
       <c r="E5" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -666,33 +742,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
+            <t>CA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -746,7 +841,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -774,33 +888,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+            <t>GC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -828,38 +961,57 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AA</t>
+            <t>TT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
       <c r="E9" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -896,19 +1048,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TC</t>
+            <t>AC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -950,19 +1121,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -1016,7 +1206,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TG</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -1044,33 +1253,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CC</t>
+            <t>AA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -1124,7 +1352,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TT</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>C</t>
           </r>
         </is>
       </c>
@@ -1166,19 +1413,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
             <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -1232,7 +1498,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GA</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -1274,19 +1559,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CA</t>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -1328,19 +1632,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
             <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>C</t>
           </r>
         </is>
       </c>
@@ -1368,33 +1691,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+            <t>AC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>C</t>
           </r>
         </is>
       </c>
@@ -1436,19 +1778,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AA</t>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -1476,7 +1837,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AT</t>
+            <t>AG</t>
           </r>
           <r>
             <rPr>
@@ -1502,7 +1863,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GT</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -1530,33 +1910,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -1598,19 +1997,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -1638,33 +2056,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+            <t>CC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -1706,19 +2143,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AT</t>
+            <t>GA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -1746,33 +2202,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
             <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -1814,19 +2289,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AT</t>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -1880,7 +2374,26 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GA</t>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -1922,19 +2435,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GC</t>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -1962,33 +2494,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>GG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>GA</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -2016,33 +2567,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TT</t>
+            <t>GG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -2070,33 +2640,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
             <t>GT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
           </r>
         </is>
       </c>
@@ -2124,33 +2713,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
             <t>GT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -2192,19 +2800,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AC</t>
+            <t>TA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -2246,19 +2873,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TC</t>
+            <t>TA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -2286,33 +2932,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+            <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>C</t>
           </r>
         </is>
       </c>
@@ -2340,33 +3005,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TG</t>
+            <t>TC</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -2408,19 +3092,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>CT</t>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>G</t>
           </r>
         </is>
       </c>
@@ -2448,33 +3151,52 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>AG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
+            <t>TT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
             <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>[</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>TG</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>]</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
           </r>
         </is>
       </c>
@@ -2485,16 +3207,16 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Del2:U2:R2</t>
+          <t>Del2:M1</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Del(2,8):U(1,2):R(2,4)</t>
+          <t>Del(2,5):M1</t>
         </is>
       </c>
       <c r="C40" s="4">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
@@ -2502,53 +3224,93 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GA</t>
+            <t>TT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <u val="double"/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>}</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>}</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GT</t>
           </r>
         </is>
       </c>
       <c r="E40" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Del2:U2:R2</t>
+          <t>Del2:M1</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Del(2,8):U(1,2):R(2,4)</t>
+          <t>Del(2,5):M1</t>
         </is>
       </c>
       <c r="C41" s="4">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
@@ -2556,33 +3318,73 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TG</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TT</t>
+            <t>AA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&lt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <u val="double"/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>}</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>A</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>}</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>AA</t>
           </r>
         </is>
       </c>
@@ -2610,7 +3412,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TT</t>
+            <t>AC</t>
           </r>
           <r>
             <rPr>
@@ -2631,7 +3433,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
+            <t>A</t>
           </r>
           <r>
             <rPr>
@@ -2645,43 +3447,43 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>G</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>A</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
             <t>}</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GT</t>
+            <t>TA</t>
           </r>
         </is>
       </c>
       <c r="E42" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -2704,7 +3506,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AA</t>
+            <t>AC</t>
           </r>
           <r>
             <rPr>
@@ -2833,7 +3635,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>G</t>
+            <t>T</t>
           </r>
           <r>
             <rPr>
@@ -2864,7 +3666,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TA</t>
+            <t>AT</t>
           </r>
         </is>
       </c>
@@ -2958,7 +3760,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AA</t>
+            <t>GC</t>
           </r>
         </is>
       </c>
@@ -2986,7 +3788,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AC</t>
+            <t>CC</t>
           </r>
           <r>
             <rPr>
@@ -3052,7 +3854,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AT</t>
+            <t>GT</t>
           </r>
         </is>
       </c>
@@ -3080,7 +3882,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AC</t>
+            <t>CC</t>
           </r>
           <r>
             <rPr>
@@ -3101,52 +3903,52 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>}</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>A</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>T</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>}</t>
           </r>
           <r>
             <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>A</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>}</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GC</t>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>GT</t>
           </r>
         </is>
       </c>
@@ -3174,7 +3976,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CC</t>
+            <t>GA</t>
           </r>
           <r>
             <rPr>
@@ -3268,7 +4070,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CC</t>
+            <t>GA</t>
           </r>
           <r>
             <rPr>
@@ -3289,52 +4091,52 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>C</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>}</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <color rgb="FFFF1493"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>T</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>C</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>}</t>
           </r>
           <r>
             <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>A</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>}</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>CA</t>
           </r>
         </is>
       </c>
@@ -3362,7 +4164,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GA</t>
+            <t>TA</t>
           </r>
           <r>
             <rPr>
@@ -3397,7 +4199,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
+            <t>C</t>
           </r>
           <r>
             <rPr>
@@ -3456,7 +4258,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GA</t>
+            <t>TC</t>
           </r>
           <r>
             <rPr>
@@ -3477,7 +4279,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>C</t>
+            <t>T</t>
           </r>
           <r>
             <rPr>
@@ -3491,38 +4293,38 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
+            <t>G</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Liberation Mono"/>
+            </rPr>
+            <t>{</t>
+          </r>
+          <r>
+            <rPr>
+              <u val="double"/>
+              <rFont val="Liberation Mono"/>
+            </rPr>
             <t>T</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>C</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
             <t>}</t>
           </r>
           <r>
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CA</t>
+            <t>AT</t>
           </r>
         </is>
       </c>
@@ -3550,7 +4352,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TA</t>
+            <t>TC</t>
           </r>
           <r>
             <rPr>
@@ -3571,7 +4373,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>A</t>
+            <t>T</t>
           </r>
           <r>
             <rPr>
@@ -3585,7 +4387,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>C</t>
+            <t>G</t>
           </r>
           <r>
             <rPr>
@@ -3604,7 +4406,7 @@
               <u val="double"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>A</t>
+            <t>T</t>
           </r>
           <r>
             <rPr>
@@ -3616,7 +4418,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>GT</t>
+            <t>CT</t>
           </r>
         </is>
       </c>
@@ -3710,7 +4512,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>AT</t>
+            <t>TA</t>
           </r>
         </is>
       </c>
@@ -3738,7 +4540,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
+            <t>TT</t>
           </r>
           <r>
             <rPr>
@@ -3759,7 +4561,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
+            <t>A</t>
           </r>
           <r>
             <rPr>
@@ -3773,7 +4575,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>G</t>
+            <t>C</t>
           </r>
           <r>
             <rPr>
@@ -3792,7 +4594,7 @@
               <u val="double"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>T</t>
+            <t>A</t>
           </r>
           <r>
             <rPr>
@@ -3804,7 +4606,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>CT</t>
+            <t>GA</t>
           </r>
         </is>
       </c>
@@ -3832,7 +4634,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TC</t>
+            <t>TT</t>
           </r>
           <r>
             <rPr>
@@ -3867,7 +4669,7 @@
               <color rgb="FFFF1493"/>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>G</t>
+            <t>C</t>
           </r>
           <r>
             <rPr>
@@ -3898,7 +4700,7 @@
             <rPr>
               <rFont val="Liberation Mono"/>
             </rPr>
-            <t>TA</t>
+            <t>GT</t>
           </r>
         </is>
       </c>
@@ -3906,202 +4708,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>Del2:M1</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>Del(2,5):M1</t>
-        </is>
-      </c>
-      <c r="C56" s="4">
-        <v>17</v>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <u val="double"/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>A</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>}</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>C</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>A</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>}</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GA</t>
-          </r>
-        </is>
-      </c>
-      <c r="E56" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>Del2:M1</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>Del(2,5):M1</t>
-        </is>
-      </c>
-      <c r="C57" s="4">
-        <v>17</v>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>TT</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&lt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <u val="double"/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>}</t>
-          </r>
-          <r>
-            <rPr>
-              <b/>
-              <color rgb="FFFF1493"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>C</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>&gt;</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>{</t>
-          </r>
-          <r>
-            <rPr>
-              <u val="double"/>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>T</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>}</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Liberation Mono"/>
-            </rPr>
-            <t>GT</t>
-          </r>
-        </is>
-      </c>
-      <c r="E57" s="4">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A2:A41"/>
-    <mergeCell ref="B2:B41"/>
-    <mergeCell ref="C2:C41"/>
-    <mergeCell ref="A42:A57"/>
-    <mergeCell ref="B42:B57"/>
-    <mergeCell ref="C42:C57"/>
+    <mergeCell ref="A2:A39"/>
+    <mergeCell ref="B2:B39"/>
+    <mergeCell ref="C2:C39"/>
+    <mergeCell ref="A40:A55"/>
+    <mergeCell ref="B40:B55"/>
+    <mergeCell ref="C40:C55"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>